<commit_message>
2026/05/22 UI, Firebase setting, table update
</commit_message>
<xml_diff>
--- a/total_df.xlsx
+++ b/total_df.xlsx
@@ -2513,22 +2513,22 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>삼겹양지</t>
+          <t>탕갈비</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>86M</t>
+          <t>86R</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>356</t>
+          <t>70</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>10,523.22</t>
+          <t>2,230.20</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2538,45 +2538,49 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>ONEYRICGA1234900</t>
+          <t>MAEU259395871</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2028.01.25</t>
+          <t>2027.08.03</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>29.56</v>
+        <v>31.86</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>SEL</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>탕갈비</t>
+          <t>삼겹양지</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>86R</t>
+          <t>86M</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>356</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>2,230.20</t>
+          <t>10,523.22</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2586,27 +2590,23 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>MAEU259395871</t>
+          <t>ONEYRICGA1234900</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2027.08.03</t>
+          <t>2028.01.25</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>31.86</v>
+        <v>29.56</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>EXCEL</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>SEL</t>
-        </is>
-      </c>
+      <c r="J44" t="inlineStr"/>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
     </row>
@@ -2765,22 +2765,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>토시살</t>
+          <t>삼겹양지</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>86E</t>
+          <t>86M</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>453</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>759.60</t>
+          <t>13,639.83</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2790,16 +2790,16 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>HDMUDALA69839800</t>
+          <t>ONEYRICFJQ530700</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2027.02.09</t>
+          <t>2027.11.07</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>16.88</v>
+        <v>30.11</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2865,22 +2865,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>삼겹양지</t>
+          <t>토시살</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>86M</t>
+          <t>86E</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>453</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>13,639.83</t>
+          <t>759.60</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -2890,16 +2890,16 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>ONEYRICFJQ530700</t>
+          <t>HDMUDALA69839800</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2027.11.07</t>
+          <t>2027.02.09</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>30.11</v>
+        <v>16.88</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -13836,7 +13836,7 @@
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>672.41</t>
+          <t>494.96</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
@@ -13856,7 +13856,7 @@
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>12.23</t>
+          <t>9.00</t>
         </is>
       </c>
       <c r="I254" t="inlineStr">
@@ -15624,7 +15624,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>417.35</t>
+          <t>314.51</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -15644,7 +15644,7 @@
       </c>
       <c r="H284" t="inlineStr">
         <is>
-          <t>27.82</t>
+          <t>20.97</t>
         </is>
       </c>
       <c r="I284" t="inlineStr">
@@ -19868,7 +19868,7 @@
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>194.82</t>
+          <t>112.81</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
@@ -19888,7 +19888,7 @@
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>12.99</t>
+          <t>7.52</t>
         </is>
       </c>
       <c r="I355" t="inlineStr">
@@ -22932,7 +22932,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>368.22</t>
+          <t>268.70</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
@@ -22952,7 +22952,7 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t>26.30</t>
+          <t>19.20</t>
         </is>
       </c>
       <c r="I406" t="inlineStr">
@@ -24366,7 +24366,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>702.50</t>
+          <t>604.87</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
@@ -24386,7 +24386,7 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t>16.30</t>
+          <t>14.07</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
@@ -24722,7 +24722,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>405.92</t>
+          <t>302.91</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
@@ -24742,7 +24742,7 @@
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t>40.59</t>
+          <t>30.29</t>
         </is>
       </c>
       <c r="I436" t="inlineStr">
@@ -25972,7 +25972,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>3,666.66</t>
+          <t>3,413.80</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
@@ -25992,7 +25992,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>28.42</t>
+          <t>26.50</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">

</xml_diff>